<commit_message>
feat(spec): finalize v3.1.0 commercial baseline with multi-defender crypto, 352h WBS, and verified CVSS suite
- Architecture: Bounded Program-Scoped Multi-Defender Model (N <= 10) with recipient_set_version concurrency guard and dual-lane payload isolation
- Cryptography: Historical-access isolation (explicitly distinguishing from forward secrecy) with audited browser-side session key re-wrapping
- WBS & Workload: Expanded commercial work packages (WP-7.1 to WP-7.9) to 88h; unified 352h total across 8 Sprints with dynamic Excel SUM formulas
- CVSS Suite: Restructured to 45 mathematically unique vectors (30 real-world NVD CVEs + 15 boundaries); corrected CVE-2021-41773 and FIRST.org Examples citation
- Verification: Built verify_cvss_engine.py (100% calculation parity) and lint_all_specifications.py (67/67 passing checks)
- Deliverables: Synchronized and recompiled BRD.docx, SRS.docx (6 embedded diagrams), and WBS.xlsx across requirements/ and Resources/
</commit_message>
<xml_diff>
--- a/requirements/WBS.xlsx
+++ b/requirements/WBS.xlsx
@@ -694,7 +694,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>264 Total Hours (236h Core + 28h Buffer / 12 Weeks = 22.0 h/wk)</t>
+          <t>352 Total Hours (264h Academic Baseline + 88h Commercial Extension)</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Commercial Baseline &amp; Academic Evaluation Specification (Version 3.0.0)</t>
+          <t>Commercial Baseline &amp; Academic Evaluation Specification (Version 3.1.0)</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2039,14 +2039,464 @@
       </c>
     </row>
     <row r="27">
-      <c r="E27" s="13" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.1</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>FR-1.3</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Auth Hardening &amp; Session Revocation</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>TOTP MFA enrollment, password reset with immediate session revocation (JWT jti blacklisting), and MFA recovery codes</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>W13–W14</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>WP-2.2</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.2</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>FR-1.4</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Guided Onboarding &amp; Domain Verification</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Step-by-step wizard: DNS TXT verification, PGP key generation, RFC 9116 download, and public program activation</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>W13–W14</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>WP-3.2</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.3</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>FR-1.5</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Private Program Access &amp; Invite Lifecycle</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Cryptographic invitation tokens (`token_hash` SHA-256 storage, 72h expiry, one-time redemption, uninvited email rejection)</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>W13–W14</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>WP-2.1</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.4</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>FR-3.6</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Multi-Defender Keying &amp; Session Re-Wrapping</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Local key export UI, program keyring versioning (`recipient_set_version`), and audited historical session-key re-wrapping</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>W15–W16</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>WP-3.4</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.5</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>FR-5.4</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Notification Outbox Worker &amp; Deduplication</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Outbox table pattern, exponential backoff retries, idempotency keys (no duplicate alerts), and minimal-metadata email templates</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>W15–W16</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>WP-5.2</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.6</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>FR-7.5</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Redacted Evidence Export Engine</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Browser-side PDF/JSON export after local decryption. Excludes free-text exploit details by default; includes full preview before download</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>W15–W16</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>WP-6.1</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.7</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>FR-8.4</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Production Cloud &amp; Stripe Subscriptions</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Stripe Checkout, Customer Portal, webhook idempotency, failed payment grace periods, cancellation downgrade, and seat entitlement checks</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>WP-1.1</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>WP-7.8</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>FR-8.5</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>MOD-7: Commercial Launch</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Disaster Recovery &amp; Incident Runbooks</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Automated daily PostgreSQL + R2 backup restore drill in sandbox, customer hard-deletion workflow, and incident response runbook</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>W17–W18</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>WP-1.2</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.9</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>GOV-02</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>GOV: Contingency &amp; Buffer</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Commercial Launch Contingency Buffer</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Buffer for unexpected billing edge cases, webhook debugging, and production pilot support</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>W13–W18</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>Taha Asadullah</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>WP-7.1</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" s="13" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED ENGINEERING HOURS:</t>
         </is>
       </c>
-      <c r="G27" s="14">
-        <f>SUM(G2:G26)</f>
-        <v>264</v>
+      <c r="G36" s="14">
+        <f>SUM(G2:G35)</f>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -2306,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2478,7 +2928,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Dual-recipient payload encryption, R2 attachment upload, CVSS 3.1 engine, in-browser decryption, basic triage</t>
+          <t>Multi-recipient payload encryption, R2 attachment upload, CVSS 3.1 engine, in-browser decryption, basic triage</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2566,14 +3016,84 @@
       </c>
     </row>
     <row r="8">
-      <c r="E8" s="13" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Weeks 13–15</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>WP-7.1, WP-7.2, WP-7.3, WP-7.4, Buffer (4h)</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>TOTP MFA, session revocation, guided onboarding wizard, tokenized private programs, multi-defender key management</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Milestone 3: Controlled Commercial Pilot</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 8</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Weeks 16–18</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>WP-7.5, WP-7.6, WP-7.7, WP-7.8, Buffer (6h)</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Notification outbox worker, redacted evidence export engine, Stripe subscription lifecycle, DR sandbox restore</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Milestone 4: Commercial Launch Gate (DoRG)</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>[ROADMAP]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>TOTAL PLANNED SPRINT HOURS:</t>
         </is>
       </c>
-      <c r="F8" s="14">
-        <f>SUM(F2:F7)</f>
-        <v>264</v>
+      <c r="F10" s="14">
+        <f>SUM(F2:F9)</f>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -2587,7 +3107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2800,13 +3320,188 @@
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="13" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Production Web Hosting</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Vercel Pro</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Custom domain, isolated team compute</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>**$20.00**</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Production Database</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Neon Serverless Launch</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>10 GB Storage, automated daily backups</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>**$19.00**</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Encrypted Storage (R2)</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Cloudflare R2 Standard</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>50 GB pooled storage baseline</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>**$0.75**</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Transactional Email</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Resend Pro</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>50,000 emails/mo, dedicated domain</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>**$20.00**</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Custom Domain &amp; DNS</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Cloudflare Registrar</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>`.com` / `.security` TLD</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>**$1.25**</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Payment Gateway</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Stripe Connect / Billing</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Automated subscription invoicing</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>**Variable**</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL FIXED INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>**Baseline for ~10–25 Active Tenants**</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>**$61.00 / month**</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>TOTAL DEMO INFRASTRUCTURE COST:</t>
         </is>
       </c>
-      <c r="E9" s="18">
-        <f>SUM(E2:E8)</f>
+      <c r="E16" s="18">
+        <f>SUM(E2:E15)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>